<commit_message>
feat: track three additional fire journals
</commit_message>
<xml_diff>
--- a/skills/fire-safety-paper-monitor/templates/journal-rss-table.xlsx
+++ b/skills/fire-safety-paper-monitor/templates/journal-rss-table.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="期刊清单" sheetId="1" r:id="rId1"/>
+    <sheet name="Journal List" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:B75"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -875,6 +875,42 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Fire and Materials</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>https://onlinelibrary.wiley.com/feed/10991018/most-recent</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Journal of Structural Fire Engineering</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>International Journal of Wildland Fire</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: track five comprehensive journals
</commit_message>
<xml_diff>
--- a/skills/fire-safety-paper-monitor/templates/journal-rss-table.xlsx
+++ b/skills/fire-safety-paper-monitor/templates/journal-rss-table.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B75"/>
+  <dimension ref="A1:B80"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -911,6 +911,66 @@
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Nature</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/nature.rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Science</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>https://www.science.org/action/showFeed?type=etoc&amp;feed=rss&amp;jc=science</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Nature Communications</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/ncomms.rss</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Proceedings of the National Academy of Sciences</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>https://www.pnas.org/action/showFeed?type=etoc&amp;feed=rss&amp;jc=pnas</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Communications Engineering</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>https://www.nature.com/commseng.rss</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>